<commit_message>
FC/GPS layout update (still rev A): MCU centred, J6 on the front edge, buck on the left edge, EMI fixes
- FC: MCU at the board centre, IMU south of it (rot 270, axes remapped in firmware), ESC link B J6 next to J5 on
  the front edge, input buck L3/U12 on the left edge (out of the corner between the rear LEDs)
- FC: LEDs D3/D4 rotated, LED supply pre-routed away from the magnetometer; EMI check script and results
- GPS: Qwiic J1 moved to v = +3.6, right above FC J3
- re-routed, DRC 0 on both boards; Gerber, STEP, PDF, BoM/CPL, views, stack check regenerated; docs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189Xg6tRAL4bRZ656VQBtPX
</commit_message>
<xml_diff>
--- a/00 - Docs/00 - FC_Docs/ACwing_FC_A_CPL.xlsx
+++ b/00 - Docs/00 - FC_Docs/ACwing_FC_A_CPL.xlsx
@@ -494,12 +494,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>21.8000mm</t>
+          <t>24.8000mm</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>27.8000mm</t>
+          <t>24.8000mm</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -544,12 +544,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>8.7196mm</t>
+          <t>4.0709mm</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>14.1567mm</t>
+          <t>10.2816mm</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
@@ -594,12 +594,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>19.0000mm</t>
+          <t>15.4000mm</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>12.7000mm</t>
+          <t>14.2000mm</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -619,12 +619,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>17.0000mm</t>
+          <t>19.5770mm</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>17.6000mm</t>
+          <t>13.2654mm</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -644,12 +644,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>22.2000mm</t>
+          <t>24.6022mm</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>30.2000mm</t>
+          <t>27.2509mm</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -669,12 +669,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>21.6000mm</t>
+          <t>24.6000mm</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>23.4000mm</t>
+          <t>20.4000mm</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>21.6000mm</t>
+          <t>24.6000mm</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>22.4000mm</t>
+          <t>19.4000mm</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>15.6000mm</t>
+          <t>11.6000mm</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>20.6000mm</t>
+          <t>21.6000mm</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>17.3000mm</t>
+          <t>13.3000mm</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0</v>
+        <v>270</v>
       </c>
     </row>
     <row r="14">
@@ -869,12 +869,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>23.0000mm</t>
+          <t>26.0000mm</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>23.9000mm</t>
+          <t>20.9000mm</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -894,12 +894,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>17.7000mm</t>
+          <t>20.7000mm</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>28.6000mm</t>
+          <t>25.6000mm</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>12.4000mm</t>
+          <t>15.4000mm</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>21.0000mm</t>
+          <t>18.0000mm</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -944,12 +944,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>21.6000mm</t>
+          <t>24.6000mm</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>20.4000mm</t>
+          <t>17.4000mm</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -969,12 +969,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>14.5500mm</t>
+          <t>17.5500mm</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>28.4000mm</t>
+          <t>25.4000mm</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>13.4736mm</t>
+          <t>16.3500mm</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>27.0196mm</t>
+          <t>24.4000mm</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>15.7500mm</t>
+          <t>18.5202mm</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>18.4000mm</t>
+          <t>15.5928mm</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1044,12 +1044,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>12.0000mm</t>
+          <t>15.0000mm</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>24.8000mm</t>
+          <t>21.8000mm</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>22.0000mm</t>
+          <t>22.9959mm</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>13.4000mm</t>
+          <t>12.5644mm</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27">
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>4.6157mm</t>
+          <t>6.2749mm</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>8.5032mm</t>
+          <t>7.0015mm</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>13.0500mm</t>
+          <t>8.2000mm</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>1.4866mm</t>
+          <t>18.1000mm</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>8.8281mm</t>
+          <t>11.0000mm</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>3.7663mm</t>
+          <t>17.2000mm</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>90</v>
+        <v>270</v>
       </c>
     </row>
     <row r="40">
@@ -1594,12 +1594,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>3.1250mm</t>
+          <t>11.8000mm</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>16.6000mm</t>
+          <t>36.8500mm</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48">
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>11.5146mm</t>
+          <t>14.5146mm</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>22.3109mm</t>
+          <t>19.3109mm</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1644,12 +1644,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>12.2500mm</t>
+          <t>15.2500mm</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>23.6866mm</t>
+          <t>20.6866mm</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>4.7019mm</t>
+          <t>3.1000mm</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>4.6511mm</t>
+          <t>15.4000mm</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>21.0000mm</t>
+          <t>13.6000mm</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>22.0000mm</t>
+          <t>13.9964mm</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>11.4000mm</t>
+          <t>9.9496mm</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="55">
@@ -1794,12 +1794,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>23.8000mm</t>
+          <t>26.8000mm</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>29.6000mm</t>
+          <t>26.6000mm</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1819,12 +1819,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>23.8000mm</t>
+          <t>26.0000mm</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>30.6000mm</t>
+          <t>27.6000mm</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>11.4000mm</t>
+          <t>14.4000mm</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>17.8000mm</t>
+          <t>14.8000mm</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -1869,12 +1869,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>11.4000mm</t>
+          <t>14.4000mm</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>16.8000mm</t>
+          <t>13.8000mm</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>21.6000mm</t>
+          <t>24.6000mm</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>21.4000mm</t>
+          <t>18.4000mm</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>25.6000mm</t>
+          <t>28.6500mm</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>22.6000mm</t>
+          <t>19.6866mm</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>25.6000mm</t>
+          <t>28.6500mm</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>23.6000mm</t>
+          <t>20.6866mm</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>22.0000mm</t>
+          <t>22.6000mm</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>18.0000mm</t>
+          <t>14.0000mm</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2044,12 +2044,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>23.0000mm</t>
+          <t>23.6000mm</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>18.0000mm</t>
+          <t>14.0000mm</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>23.4000mm</t>
+          <t>26.4000mm</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>25.6000mm</t>
+          <t>22.6000mm</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2094,12 +2094,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>23.9832mm</t>
+          <t>26.9832mm</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>24.0524mm</t>
+          <t>21.0524mm</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>23.4000mm</t>
+          <t>26.4000mm</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>26.6000mm</t>
+          <t>23.6000mm</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>23.4000mm</t>
+          <t>26.4000mm</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>27.6000mm</t>
+          <t>24.6000mm</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2169,12 +2169,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>10.6063mm</t>
+          <t>13.6063mm</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>24.3003mm</t>
+          <t>21.3003mm</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2194,12 +2194,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>19.1000mm</t>
+          <t>14.6000mm</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>28.6000mm</t>
+          <t>28.0000mm</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>18.1250mm</t>
+          <t>14.6000mm</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>29.9929mm</t>
+          <t>29.0000mm</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -2244,12 +2244,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>10.9500mm</t>
+          <t>13.5391mm</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>20.5134mm</t>
+          <t>27.0002mm</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2269,12 +2269,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>19.8000mm</t>
+          <t>16.2000mm</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>30.0000mm</t>
+          <t>29.2000mm</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -2283,7 +2283,7 @@
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
     </row>
     <row r="75">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>22.0000mm</t>
+          <t>21.6281mm</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>15.0000mm</t>
+          <t>15.1472mm</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
     </row>
     <row r="77">
@@ -2344,12 +2344,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>17.4243mm</t>
+          <t>17.6000mm</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>15.6263mm</t>
+          <t>12.2000mm</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2358,7 +2358,7 @@
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
     </row>
     <row r="78">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>18.8000mm</t>
+          <t>17.5514mm</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>13.6000mm</t>
+          <t>14.2333mm</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2469,12 +2469,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>12.9213mm</t>
+          <t>10.4000mm</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>7.2671mm</t>
+          <t>14.0000mm</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="83">
@@ -2494,12 +2494,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>14.1621mm</t>
+          <t>11.4000mm</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>6.3212mm</t>
+          <t>14.0000mm</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -2508,7 +2508,7 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="84">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>16.4000mm</t>
+          <t>12.4000mm</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="85">
@@ -2544,12 +2544,12 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>17.0000mm</t>
+          <t>20.0000mm</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>23.0000mm</t>
+          <t>20.0000mm</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -2619,12 +2619,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>19.0000mm</t>
+          <t>15.4000mm</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>11.0000mm</t>
+          <t>12.2000mm</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>16.0000mm</t>
+          <t>19.0000mm</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>29.0745mm</t>
+          <t>26.0745mm</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -2694,12 +2694,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>26.8687mm</t>
+          <t>28.9319mm</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>16.3973mm</t>
+          <t>16.4271mm</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>11.2645mm</t>
+          <t>7.9000mm</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>4.8243mm</t>
+          <t>15.0000mm</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -2769,12 +2769,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>11.4000mm</t>
+          <t>14.4000mm</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>25.4000mm</t>
+          <t>22.4000mm</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">

</xml_diff>

<commit_message>
FC rev A: CPL fixes from the JLC placement preview
- Bottom side: rotation = 180 - KiCad rotation + correction (JLC mirrors
  bottom parts about the Y axis); U10, U11, U13 were 90/180 deg off.
- Corrections: U10 WSON-8 270, U13 SOT-353 180, U12 VSON-10 0 (was 270),
  LEDs D1-D4 (XL-2020) 180.
- J1 USB-C: CPL position moved 1.46 mm toward the pins (JLC origin = pad-area
  centre, KiCad origin = body centre).
- README: CPL notes and checks updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189Xg6tRAL4bRZ656VQBtPX
</commit_message>
<xml_diff>
--- a/00 - Docs/00 - FC_Docs/ACwing_FC_A_CPL.xlsx
+++ b/00 - Docs/00 - FC_Docs/ACwing_FC_A_CPL.xlsx
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9">
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11">
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15">
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21">
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22">
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23">
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>270</v>
+        <v>90</v>
       </c>
     </row>
     <row r="39">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>270</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>35.7670mm</t>
+          <t>34.7346mm</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>4.2330mm</t>
+          <t>5.2654mm</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50">
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56">
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="57">
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="58">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59">
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="60">
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="62">
@@ -1983,7 +1983,7 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="63">
@@ -2008,7 +2008,7 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64">
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="67">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="69">
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="70">
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="72">
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="73">
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="74">
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="79">
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="82">
@@ -2708,7 +2708,7 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="92">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>270</v>
+        <v>90</v>
       </c>
     </row>
     <row r="93">
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="94">
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">

</xml_diff>